<commit_message>
two test case added
</commit_message>
<xml_diff>
--- a/testData/Opencart_LoginData.xlsx
+++ b/testData/Opencart_LoginData.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{EE676F4B-BE0F-4CA0-92AA-B891C694F05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{EAF8F34D-7B1B-4996-9D28-472FA2B0DB43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1F2D179E-37D2-4BC0-88A9-F5C135B87DA5}"/>
   </bookViews>
@@ -16,21 +16,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
   <si>
     <t>username</t>
   </si>
@@ -75,6 +66,9 @@
   </si>
   <si>
     <t>shami@08</t>
+  </si>
+  <si>
+    <t>toji123@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -559,6 +553,9 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="21" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B7" s="4" t="s">
         <v>11</v>
       </c>
@@ -576,8 +573,9 @@
     <hyperlink ref="A6" r:id="rId6" xr:uid="{75A4F8D6-7BF1-446B-9367-475FA4FB44C7}"/>
     <hyperlink ref="B6" r:id="rId7" xr:uid="{01D5649A-5E55-45E1-9B81-1CE430C208A1}"/>
     <hyperlink ref="B7" r:id="rId8" xr:uid="{A49E65D7-8AA3-4B9D-BC07-4CDF7ACB2B0E}"/>
+    <hyperlink ref="A7" r:id="rId9" xr:uid="{6C16F375-D6FB-4D81-9429-60C1A0E446A2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId9"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>